<commit_message>
[add] 프로토타입용 Character관련 json과 CharacterData 준비
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Character.xlsx
+++ b/JsonConverter/ExcelFiles/Character.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fileVersion appName="HCell" lastEdited="12.0" lowestEdited="12.0" rupBuild="0.535"/>
+  <x:fileVersion appName="HCell" lastEdited="10.0" lowestEdited="10.0" rupBuild="0.12458"/>
   <x:workbookPr date1904="0" showBorderUnselectedTables="1" filterPrivacy="0" promptedSolutions="0" showInkAnnotation="1" backupFile="0" saveExternalLinkValues="1" codeName="ThisWorkbook" hidePivotFieldList="0" allowRefreshQuery="0" publishItems="0" checkCompatibility="0" autoCompressPictures="1" refreshAllConnections="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_NRUnityProjects\UnityBasic_6\JsonConverter\ExcelFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\0_NRUnityProjects\Boxing_or_IdleGame\JsonConverter\ExcelFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <x:bookViews>
-    <x:workbookView xWindow="0" yWindow="0" windowWidth="21390" windowHeight="15240"/>
+    <x:workbookView xWindow="0" yWindow="0" windowWidth="28545" windowHeight="11745"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="DNTable_Character&lt;Hero&gt;" sheetId="1" r:id="rId4"/>
@@ -19,160 +19,61 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <x:si>
-    <x:t>skill_fireball_01,skill_normalSword_01</x:t>
+    <x:t>Atk</x:t>
   </x:si>
   <x:si>
-    <x:t>마키나코르</x:t>
+    <x:t>float</x:t>
   </x:si>
   <x:si>
-    <x:t>사피크로우</x:t>
+    <x:t>기본 적이다</x:t>
   </x:si>
   <x:si>
-    <x:t>오즈마</x:t>
+    <x:t>Def</x:t>
   </x:si>
   <x:si>
-    <x:t>character_machinacor_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_sapicrow_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BaseStatDataId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>도로트비아</x:t>
-  </x:si>
-  <x:si>
-    <x:t>소환 마법을 사용할 수 있는 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_CoffeeCup_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 별로 무기가 고정인 경우용</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Braclet_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_daniel_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>모든 마법을 사용할 수 있는 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_victor_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_ozma_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>방문자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Costume_03</x:t>
+    <x:t>Id</x:t>
   </x:si>
   <x:si>
     <x:t>캐릭터 고유 ID</x:t>
   </x:si>
   <x:si>
-    <x:t>SkillList</x:t>
-  </x:si>
-  <x:si>
-    <x:t>UseWeaponId</x:t>
-  </x:si>
-  <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
-    <x:t>잉여로운 버프 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>BasicCostumeId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Weapon_Sword_1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>캐릭터 전체 컨셉이나 스토리</x:t>
-  </x:si>
-  <x:si>
-    <x:t>헬레나</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>스킬</x:t>
-  </x:si>
-  <x:si>
-    <x:t>다니엘</x:t>
-  </x:si>
-  <x:si>
-    <x:t>빅토르</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_hellena_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_rest_coffee_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>skill_normalSword_01</x:t>
+    <x:t>기본 캐릭터이다</x:t>
   </x:si>
   <x:si>
     <x:t>Name</x:t>
   </x:si>
   <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
     <x:t>string</x:t>
   </x:si>
   <x:si>
-    <x:t>(name)</x:t>
+    <x:t>character_01</x:t>
   </x:si>
   <x:si>
-    <x:t>오즈의 세계에 존재하는 궁극의 캐릭터</x:t>
+    <x:t>김기본</x:t>
   </x:si>
   <x:si>
-    <x:t>character_valentileaon_01</x:t>
+    <x:t>Hp</x:t>
   </x:si>
   <x:si>
-    <x:t>stat_dummy_01</x:t>
+    <x:t>김적</x:t>
   </x:si>
   <x:si>
-    <x:t>도로트비아 학파를 설립한 영웅 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_ozbasic_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>마키나코르 학파를 설립한 영웅 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>발렌티레온</x:t>
-  </x:si>
-  <x:si>
-    <x:t>사피크로우 학파를 설립한 영웅 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>발렌티레온 학파를 설립한 영웅 캐릭터</x:t>
-  </x:si>
-  <x:si>
-    <x:t>character_dorothvia_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>오즈의 세계에 처음 들어온 방문자</x:t>
-  </x:si>
-  <x:si>
-    <x:t>stat_basicCharacter_01</x:t>
+    <x:t>opponent_01</x:t>
   </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="9">
+  <x:fonts count="8">
     <x:font>
       <x:name val="Arial"/>
       <x:sz val="10"/>
@@ -204,17 +105,12 @@
       <x:color rgb="ff000000"/>
     </x:font>
     <x:font>
-      <x:name val="&quot;맑은 고딕&quot;"/>
+      <x:name val="맑은 고딕"/>
       <x:sz val="10"/>
       <x:color rgb="ff000000"/>
     </x:font>
     <x:font>
       <x:name val="맑은 고딕"/>
-      <x:sz val="10"/>
-      <x:color rgb="ff000000"/>
-    </x:font>
-    <x:font>
-      <x:name val="&quot;맑은 고딕&quot;"/>
       <x:sz val="11"/>
       <x:color rgb="ff008000"/>
     </x:font>
@@ -230,6 +126,12 @@
       <x:patternFill patternType="solid">
         <x:fgColor rgb="ffffffff"/>
         <x:bgColor indexed="64"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="ffd2f2db"/>
+        <x:bgColor rgb="ffc6efce"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -253,12 +155,6 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="ffd2f2db"/>
-        <x:bgColor rgb="ffc6efce"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="ffd2f2db"/>
         <x:bgColor indexed="64"/>
       </x:patternFill>
     </x:fill>
@@ -266,16 +162,16 @@
   <x:borders count="3">
     <x:border>
       <x:left>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:left>
       <x:right>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:right>
       <x:top>
         <x:color auto="1"/>
       </x:top>
       <x:bottom>
-        <x:color rgb="ff000000"/>
+        <x:color auto="1"/>
       </x:bottom>
     </x:border>
     <x:border>
@@ -312,64 +208,435 @@
       <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
+  <x:cellXfs count="8">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:alignment horizontal="general" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="general" vertical="bottom"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="bottom"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="표준" xfId="0" builtinId="0"/>
   </x:cellStyles>
-  <x:dxfs count="0"/>
-  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <x:dxfs count="12">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:color rgb="ff000000"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ffd7dff4"/>
+              <x:bgColor rgb="ffd7dff4"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:left style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:left>
+            <x:right style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:right>
+            <x:top style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:top>
+            <x:bottom style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:bottom>
+            <x:vertical style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:vertical>
+            <x:horizontal style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:horizontal>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:color rgb="ff000000"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ffd7dff4"/>
+              <x:bgColor rgb="ffd7dff4"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:left style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:left>
+            <x:right style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:right>
+            <x:top style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:top>
+            <x:bottom style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:bottom>
+            <x:vertical style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:vertical>
+            <x:horizontal style="thin">
+              <x:color rgb="ffffffff"/>
+            </x:horizontal>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <x:dxf/>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:fgColor rgb="ffaebfea"/>
+          <x:bgColor rgb="ffaebfea"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:top style="thick">
+              <x:color rgb="ffffffff"/>
+            </x:top>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:top style="thick">
+              <x:color rgb="ffffffff"/>
+            </x:top>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:bottom style="thick">
+              <x:color rgb="ffffffff"/>
+            </x:bottom>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:color rgb="ffffffff"/>
+            <x:b val="1"/>
+          </x:font>
+          <x:fill>
+            <x:patternFill patternType="solid">
+              <x:fgColor rgb="ff6182d6"/>
+              <x:bgColor rgb="ff6182d6"/>
+            </x:patternFill>
+          </x:fill>
+          <x:border>
+            <x:bottom style="thick">
+              <x:color rgb="ffffffff"/>
+            </x:bottom>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:color rgb="ff000000"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:border>
+            <x:left>
+              <x:color auto="1"/>
+            </x:left>
+            <x:right>
+              <x:color auto="1"/>
+            </x:right>
+            <x:top style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:top>
+            <x:bottom style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:bottom>
+            <x:vertical>
+              <x:color auto="1"/>
+            </x:vertical>
+            <x:horizontal>
+              <x:color auto="1"/>
+            </x:horizontal>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:color rgb="ff000000"/>
+          </x:font>
+          <x:border>
+            <x:left>
+              <x:color auto="1"/>
+            </x:left>
+            <x:right>
+              <x:color auto="1"/>
+            </x:right>
+            <x:top style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:top>
+            <x:bottom style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:bottom>
+            <x:vertical>
+              <x:color auto="1"/>
+            </x:vertical>
+            <x:horizontal>
+              <x:color auto="1"/>
+            </x:horizontal>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:fgColor rgb="ff94a5df"/>
+          <x:bgColor rgb="ff94a5df"/>
+        </x:patternFill>
+      </x:fill>
+      <x:border>
+        <x:top style="thin">
+          <x:color rgb="ff6182d6"/>
+        </x:top>
+        <x:bottom style="thin">
+          <x:color rgb="ff6182d6"/>
+        </x:bottom>
+      </x:border>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:fgColor rgb="ff6182d6"/>
+          <x:bgColor rgb="ff6182d6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:b val="1"/>
+          </x:font>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:border>
+            <x:top style="thin">
+              <x:color rgb="ff6182d6"/>
+            </x:top>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:b val="1"/>
+          </x:font>
+          <x:border>
+            <x:top style="thin">
+              <x:color rgb="ff6182d6"/>
+            </x:top>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:hs="http://schemas.haansoft.com/office/spreadsheet/8.0" Requires="hs">
+        <x:dxf hs:applyExtension="1">
+          <x:font hs:extension="1">
+            <x:b val="1"/>
+            <hs:useFontSpace val="0"/>
+            <hs:size val="0"/>
+            <hs:ratio val="0"/>
+            <hs:spacing val="0"/>
+            <hs:offset val="0"/>
+          </x:font>
+          <x:border>
+            <x:bottom style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:bottom>
+          </x:border>
+        </x:dxf>
+      </mc:Choice>
+      <mc:Fallback>
+        <x:dxf>
+          <x:font>
+            <x:b val="1"/>
+          </x:font>
+          <x:border>
+            <x:bottom style="medium">
+              <x:color rgb="ff6182d6"/>
+            </x:bottom>
+          </x:border>
+        </x:dxf>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </x:dxfs>
+  <x:tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <x:tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="9">
+      <x:tableStyleElement type="wholeTable" size="1" dxfId="0"/>
+      <x:tableStyleElement type="headerRow" size="1" dxfId="5"/>
+      <x:tableStyleElement type="totalRow" size="1" dxfId="4"/>
+      <x:tableStyleElement type="firstColumn" size="1" dxfId="3"/>
+      <x:tableStyleElement type="lastColumn" size="1" dxfId="3"/>
+      <x:tableStyleElement type="firstRowStripe" size="1" dxfId="2"/>
+      <x:tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
+      <x:tableStyleElement type="firstColumnStripe" size="1" dxfId="2"/>
+      <x:tableStyleElement type="secondColumnStripe" size="1" dxfId="1"/>
+    </x:tableStyle>
+    <x:tableStyle name="Light Style 1 - Accent 1" pivot="1" table="0" count="8">
+      <x:tableStyleElement type="wholeTable" size="1" dxfId="6"/>
+      <x:tableStyleElement type="headerRow" size="1" dxfId="11"/>
+      <x:tableStyleElement type="totalRow" size="1" dxfId="10"/>
+      <x:tableStyleElement type="firstColumn" size="1" dxfId="9"/>
+      <x:tableStyleElement type="lastColumn" size="1" dxfId="9"/>
+      <x:tableStyleElement type="firstRowStripe" size="1" dxfId="7"/>
+      <x:tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
+      <x:tableStyleElement type="firstColumnStripe" size="1" dxfId="8"/>
+    </x:tableStyle>
+  </x:tableStyles>
 </x:styleSheet>
 </file>
 
@@ -569,487 +836,238 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetPr codeName="Sheet1">
-    <x:outlinePr applyStyles="0" summaryBelow="0" summaryRight="1" showOutlineSymbols="1"/>
-  </x:sheetPr>
-  <x:dimension ref="A1:O35"/>
+  <x:sheetPr codeName="Sheet1"/>
+  <x:dimension ref="A1:F35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
-    <x:col min="1" max="1" width="25.4296875" style="3" customWidth="1"/>
-    <x:col min="2" max="2" width="19.54296875" style="3" customWidth="1"/>
-    <x:col min="3" max="3" width="50.7265625" style="3" customWidth="1"/>
-    <x:col min="4" max="4" width="20.26953125" style="3" customWidth="1"/>
-    <x:col min="5" max="5" width="30.54296875" style="3" customWidth="1"/>
-    <x:col min="6" max="6" width="26.54296875" style="3" customWidth="1"/>
-    <x:col min="7" max="7" width="20" style="3" customWidth="1"/>
-    <x:col min="8" max="16384" width="12.54296875" style="3"/>
+    <x:col min="1" max="1" width="25.4296875" style="1" customWidth="1"/>
+    <x:col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
+    <x:col min="3" max="3" width="50.7265625" style="1" customWidth="1"/>
+    <x:col min="4" max="4" width="20.26953125" style="1" customWidth="1"/>
+    <x:col min="5" max="5" width="30.54296875" style="1" customWidth="1"/>
+    <x:col min="6" max="6" width="26.54296875" style="1" customWidth="1"/>
+    <x:col min="7" max="7" width="20" style="1" customWidth="1"/>
+    <x:col min="8" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5" ht="15.75" customHeight="1">
+    <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B1" s="1"/>
-      <x:c r="C1" s="1" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="D1" s="2" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="E1" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
         <x:v>10</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:6" ht="13.19999999999999928946">
-      <x:c r="A2" s="1" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>35</x:v>
-      </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>35</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>35</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:7" s="13" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="12" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B3" s="12" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="C3" s="12" t="s">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="D3" s="14" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="E3" s="14" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F3" s="15" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="G3" s="13" t="s">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6" s="7" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="s">
         <x:v>6</x:v>
       </x:c>
-    </x:row>
-    <x:row r="4" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A4" s="4" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B4" s="4" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C4" s="4" t="s">
+      <x:c r="D3" s="7" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="s">
+      <x:c r="E3" s="7" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E4" s="5" t="s">
+      <x:c r="F3" s="7" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A4" s="3" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F4" s="16" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H4" s="5"/>
-      <x:c r="I4" s="5"/>
-      <x:c r="J4" s="5"/>
-      <x:c r="K4" s="5"/>
-      <x:c r="L4" s="5"/>
-      <x:c r="M4" s="5"/>
-      <x:c r="N4" s="5"/>
-      <x:c r="O4" s="5"/>
-    </x:row>
-    <x:row r="5" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A5" s="4" t="s">
+      <x:c r="B4" s="3" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C4" s="3" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="1">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E4" s="1">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F4" s="4">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6" ht="15.75" customHeight="1">
+      <x:c r="A5" s="3" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B5" s="5" t="s">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="B5" s="6" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="E5" s="5" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="F5" s="5"/>
-      <x:c r="G5" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H5" s="5"/>
-      <x:c r="I5" s="5"/>
-      <x:c r="J5" s="5"/>
-      <x:c r="K5" s="5"/>
-      <x:c r="L5" s="5"/>
-      <x:c r="M5" s="5"/>
-      <x:c r="N5" s="5"/>
-      <x:c r="O5" s="5"/>
-    </x:row>
-    <x:row r="6" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A6" s="6" t="s">
+      <x:c r="C5" s="5" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D5" s="1">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="E5" s="1">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B6" s="6" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E6" s="5" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F6" s="5"/>
-      <x:c r="G6" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H6" s="5"/>
-      <x:c r="I6" s="5"/>
-      <x:c r="J6" s="5"/>
-      <x:c r="K6" s="5"/>
-      <x:c r="L6" s="5"/>
-      <x:c r="M6" s="5"/>
-      <x:c r="N6" s="5"/>
-      <x:c r="O6" s="5"/>
-    </x:row>
-    <x:row r="7" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A7" s="4" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E7" s="5"/>
-      <x:c r="F7" s="5"/>
-      <x:c r="G7" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H7" s="5"/>
-      <x:c r="I7" s="5"/>
-      <x:c r="J7" s="5"/>
-      <x:c r="K7" s="5"/>
-      <x:c r="L7" s="5"/>
-      <x:c r="M7" s="5"/>
-      <x:c r="N7" s="5"/>
-      <x:c r="O7" s="5"/>
-    </x:row>
-    <x:row r="8" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A8" s="4" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B8" s="4" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C8" s="4" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E8" s="5"/>
-      <x:c r="F8" s="5"/>
-      <x:c r="G8" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H8" s="5"/>
-      <x:c r="I8" s="5"/>
-      <x:c r="J8" s="5"/>
-      <x:c r="K8" s="5"/>
-      <x:c r="L8" s="5"/>
-      <x:c r="M8" s="5"/>
-      <x:c r="N8" s="5"/>
-      <x:c r="O8" s="5"/>
-    </x:row>
-    <x:row r="9" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A9" s="4" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B9" s="4" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="4" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E9" s="5"/>
-      <x:c r="F9" s="5"/>
-      <x:c r="G9" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H9" s="5"/>
-      <x:c r="I9" s="5"/>
-      <x:c r="J9" s="5"/>
-      <x:c r="K9" s="5"/>
-      <x:c r="L9" s="5"/>
-      <x:c r="M9" s="5"/>
-      <x:c r="N9" s="5"/>
-      <x:c r="O9" s="5"/>
-    </x:row>
-    <x:row r="10" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A10" s="1" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="B10" s="1" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="C10" s="1" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E10" s="5"/>
-      <x:c r="F10" s="5"/>
-      <x:c r="G10" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H10" s="5"/>
-      <x:c r="I10" s="5"/>
-      <x:c r="J10" s="5"/>
-      <x:c r="K10" s="5"/>
-      <x:c r="L10" s="5"/>
-      <x:c r="M10" s="5"/>
-      <x:c r="N10" s="5"/>
-      <x:c r="O10" s="5"/>
-    </x:row>
-    <x:row r="11" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A11" s="1" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="B11" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C11" s="1" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="D11" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E11" s="5"/>
-      <x:c r="F11" s="5"/>
-      <x:c r="G11" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H11" s="5"/>
-      <x:c r="I11" s="5"/>
-      <x:c r="J11" s="5"/>
-      <x:c r="K11" s="5"/>
-      <x:c r="L11" s="5"/>
-      <x:c r="M11" s="5"/>
-      <x:c r="N11" s="5"/>
-      <x:c r="O11" s="5"/>
-    </x:row>
-    <x:row r="12" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A12" s="7" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="B12" s="7" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="D12" s="5" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="E12" s="5"/>
-      <x:c r="F12" s="5"/>
-      <x:c r="G12" s="5" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="H12" s="5"/>
-      <x:c r="I12" s="5"/>
-      <x:c r="J12" s="5"/>
-      <x:c r="K12" s="5"/>
-      <x:c r="L12" s="5"/>
-      <x:c r="M12" s="5"/>
-      <x:c r="N12" s="5"/>
-      <x:c r="O12" s="5"/>
-    </x:row>
-    <x:row r="13" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A13" s="4"/>
-      <x:c r="B13" s="4"/>
-      <x:c r="C13" s="4"/>
-      <x:c r="D13" s="5"/>
-      <x:c r="E13" s="5"/>
-      <x:c r="F13" s="5"/>
-      <x:c r="G13" s="5"/>
-      <x:c r="H13" s="5"/>
-      <x:c r="I13" s="5"/>
-      <x:c r="J13" s="5"/>
-      <x:c r="K13" s="5"/>
-      <x:c r="L13" s="5"/>
-      <x:c r="M13" s="5"/>
-      <x:c r="N13" s="5"/>
-      <x:c r="O13" s="5"/>
-    </x:row>
-    <x:row r="14" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A14" s="1"/>
-      <x:c r="B14" s="1"/>
-      <x:c r="C14" s="1"/>
-      <x:c r="D14" s="5"/>
-      <x:c r="E14" s="5"/>
-      <x:c r="F14" s="5"/>
-      <x:c r="G14" s="5"/>
-      <x:c r="H14" s="5"/>
-      <x:c r="I14" s="5"/>
-      <x:c r="J14" s="5"/>
-      <x:c r="K14" s="5"/>
-      <x:c r="L14" s="5"/>
-      <x:c r="M14" s="5"/>
-      <x:c r="N14" s="5"/>
-      <x:c r="O14" s="5"/>
-    </x:row>
-    <x:row r="15" spans="1:15" ht="15.75" customHeight="1">
-      <x:c r="A15" s="1"/>
-      <x:c r="B15" s="1"/>
-      <x:c r="C15" s="1"/>
-      <x:c r="D15" s="5"/>
-      <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5"/>
-      <x:c r="G15" s="5"/>
-      <x:c r="H15" s="5"/>
-      <x:c r="I15" s="5"/>
-      <x:c r="J15" s="5"/>
-      <x:c r="K15" s="5"/>
-      <x:c r="L15" s="5"/>
-      <x:c r="M15" s="5"/>
-      <x:c r="N15" s="5"/>
-      <x:c r="O15" s="5"/>
-    </x:row>
+      <x:c r="F5" s="1">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A6" s="5"/>
+      <x:c r="B6" s="5"/>
+      <x:c r="C6" s="5"/>
+    </x:row>
+    <x:row r="7" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A7" s="5"/>
+      <x:c r="B7" s="5"/>
+      <x:c r="C7" s="5"/>
+    </x:row>
+    <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A8" s="5"/>
+      <x:c r="B8" s="5"/>
+      <x:c r="C8" s="5"/>
+    </x:row>
+    <x:row r="9" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A9" s="5"/>
+      <x:c r="B9" s="5"/>
+      <x:c r="C9" s="5"/>
+    </x:row>
+    <x:row r="10" ht="15.75" customHeight="1"/>
+    <x:row r="11" ht="15.75" customHeight="1"/>
+    <x:row r="12" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A12" s="6"/>
+      <x:c r="B12" s="6"/>
+      <x:c r="C12" s="6"/>
+    </x:row>
+    <x:row r="13" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A13" s="3"/>
+      <x:c r="B13" s="3"/>
+      <x:c r="C13" s="3"/>
+    </x:row>
+    <x:row r="14" ht="15.75" customHeight="1"/>
+    <x:row r="15" ht="15.75" customHeight="1"/>
     <x:row r="16" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A16" s="8"/>
-      <x:c r="B16" s="8"/>
-      <x:c r="C16" s="8"/>
+      <x:c r="A16" s="5"/>
+      <x:c r="B16" s="5"/>
+      <x:c r="C16" s="5"/>
     </x:row>
     <x:row r="17" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A17" s="9"/>
-      <x:c r="B17" s="9"/>
-      <x:c r="C17" s="9"/>
+      <x:c r="A17" s="5"/>
+      <x:c r="B17" s="5"/>
+      <x:c r="C17" s="5"/>
     </x:row>
     <x:row r="18" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A18" s="9"/>
-      <x:c r="B18" s="9"/>
-      <x:c r="C18" s="9"/>
-    </x:row>
-    <x:row r="19" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A19" s="9"/>
-      <x:c r="B19" s="9"/>
-      <x:c r="C19" s="9"/>
-      <x:c r="D19" s="5"/>
-      <x:c r="E19" s="5"/>
+      <x:c r="A18" s="5"/>
+      <x:c r="B18" s="5"/>
+      <x:c r="C18" s="5"/>
+    </x:row>
+    <x:row r="19" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A19" s="5"/>
+      <x:c r="B19" s="5"/>
+      <x:c r="C19" s="5"/>
     </x:row>
     <x:row r="20" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A20" s="9"/>
-      <x:c r="B20" s="9"/>
-      <x:c r="C20" s="9"/>
+      <x:c r="A20" s="5"/>
+      <x:c r="B20" s="5"/>
+      <x:c r="C20" s="5"/>
     </x:row>
     <x:row r="21" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A21" s="9"/>
-      <x:c r="B21" s="9"/>
-      <x:c r="C21" s="9"/>
+      <x:c r="A21" s="5"/>
+      <x:c r="B21" s="5"/>
+      <x:c r="C21" s="5"/>
     </x:row>
     <x:row r="22" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A22" s="9"/>
-      <x:c r="B22" s="9"/>
-      <x:c r="C22" s="9"/>
+      <x:c r="A22" s="5"/>
+      <x:c r="B22" s="5"/>
+      <x:c r="C22" s="5"/>
     </x:row>
     <x:row r="23" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A23" s="9"/>
-      <x:c r="B23" s="9"/>
-      <x:c r="C23" s="9"/>
+      <x:c r="A23" s="5"/>
+      <x:c r="B23" s="5"/>
+      <x:c r="C23" s="5"/>
     </x:row>
     <x:row r="24" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A24" s="9"/>
-      <x:c r="B24" s="9"/>
-      <x:c r="C24" s="9"/>
-    </x:row>
-    <x:row r="25" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A25" s="9"/>
-      <x:c r="B25" s="9"/>
-      <x:c r="C25" s="9"/>
-      <x:c r="E25" s="5"/>
-    </x:row>
-    <x:row r="26" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A26" s="10"/>
-      <x:c r="B26" s="10"/>
-      <x:c r="C26" s="10"/>
-      <x:c r="E26" s="5"/>
-    </x:row>
-    <x:row r="27" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A27" s="10"/>
-      <x:c r="B27" s="10"/>
-      <x:c r="C27" s="10"/>
-      <x:c r="E27" s="5"/>
-    </x:row>
-    <x:row r="28" spans="1:5" ht="15.75" customHeight="1">
-      <x:c r="A28" s="10"/>
-      <x:c r="B28" s="10"/>
-      <x:c r="C28" s="10"/>
-      <x:c r="E28" s="5"/>
+      <x:c r="A24" s="5"/>
+      <x:c r="B24" s="5"/>
+      <x:c r="C24" s="5"/>
+    </x:row>
+    <x:row r="25" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A25" s="5"/>
+      <x:c r="B25" s="5"/>
+      <x:c r="C25" s="5"/>
+    </x:row>
+    <x:row r="26" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A26" s="6"/>
+      <x:c r="B26" s="6"/>
+      <x:c r="C26" s="6"/>
+    </x:row>
+    <x:row r="27" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A27" s="6"/>
+      <x:c r="B27" s="6"/>
+      <x:c r="C27" s="6"/>
+    </x:row>
+    <x:row r="28" spans="1:3" ht="15.75" customHeight="1">
+      <x:c r="A28" s="6"/>
+      <x:c r="B28" s="6"/>
+      <x:c r="C28" s="6"/>
     </x:row>
     <x:row r="29" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A29" s="10"/>
-      <x:c r="B29" s="10"/>
-      <x:c r="C29" s="10"/>
+      <x:c r="A29" s="6"/>
+      <x:c r="B29" s="6"/>
+      <x:c r="C29" s="6"/>
     </x:row>
     <x:row r="30" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A30" s="10"/>
-      <x:c r="B30" s="10"/>
-      <x:c r="C30" s="10"/>
+      <x:c r="A30" s="6"/>
+      <x:c r="B30" s="6"/>
+      <x:c r="C30" s="6"/>
     </x:row>
     <x:row r="31" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A31" s="10"/>
-      <x:c r="B31" s="10"/>
-      <x:c r="C31" s="10"/>
+      <x:c r="A31" s="6"/>
+      <x:c r="B31" s="6"/>
+      <x:c r="C31" s="6"/>
     </x:row>
     <x:row r="32" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A32" s="11"/>
-      <x:c r="B32" s="11"/>
-      <x:c r="C32" s="11"/>
+      <x:c r="A32" s="3"/>
+      <x:c r="B32" s="3"/>
+      <x:c r="C32" s="3"/>
     </x:row>
     <x:row r="33" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A33" s="11"/>
-      <x:c r="B33" s="11"/>
-      <x:c r="C33" s="11"/>
+      <x:c r="A33" s="3"/>
+      <x:c r="B33" s="3"/>
+      <x:c r="C33" s="3"/>
     </x:row>
     <x:row r="34" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A34" s="11"/>
-      <x:c r="B34" s="11"/>
-      <x:c r="C34" s="11"/>
+      <x:c r="A34" s="3"/>
+      <x:c r="B34" s="3"/>
+      <x:c r="C34" s="3"/>
     </x:row>
     <x:row r="35" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A35" s="11"/>
-      <x:c r="B35" s="11"/>
-      <x:c r="C35" s="11"/>
+      <x:c r="A35" s="3"/>
+      <x:c r="B35" s="3"/>
+      <x:c r="C35" s="3"/>
     </x:row>
     <x:row r="36" ht="15.75" customHeight="1"/>
     <x:row r="37" ht="15.75" customHeight="1"/>
@@ -2017,7 +2035,7 @@
     <x:row r="999" ht="15.75" customHeight="1"/>
     <x:row r="1000" ht="15.75" customHeight="1"/>
   </x:sheetData>
-  <x:pageMargins left="0.69986110925674438477" right="0.69986110925674438477" top="0.75" bottom="0.75" header="0.30000001192092895508" footer="0.30000001192092895508"/>
+  <x:pageMargins left="0.69972223043441772" right="0.69972223043441772" top="0.75" bottom="0.75" header="0.30000001192092896" footer="0.30000001192092896"/>
   <x:pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" useFirstPageNumber="0" horizontalDpi="600" verticalDpi="600" copies="1"/>
 </x:worksheet>
 </file>
</xml_diff>